<commit_message>
Add 7 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 45
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-expertise.report.xlsx
+++ b/tools/importer/reports/import-expertise.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>_reportFile</t>
   </si>
@@ -73,13 +73,34 @@
     <t>expertise</t>
   </si>
   <si>
-    <t>2026-10-02T13:38:21.376Z</t>
+    <t>2026-10-02T15:47:14.777Z</t>
   </si>
   <si>
     <t>Artificial Intelligence</t>
   </si>
   <si>
     <t>https://www.boozallen.com/expertise/artificial-intelligence.html</t>
+  </si>
+  <si>
+    <t>markets/defense/ai-for-military.report.json</t>
+  </si>
+  <si>
+    <t>["hero-banner","columns-subnav","cards-carousel","cards-horizontal","columns-backdrop","embed-marketo","columns-cta"]</t>
+  </si>
+  <si>
+    <t>markets/defense/ai-for-military</t>
+  </si>
+  <si>
+    <t>defense</t>
+  </si>
+  <si>
+    <t>2026-10-02T15:47:01.393Z</t>
+  </si>
+  <si>
+    <t>AI for Defense</t>
+  </si>
+  <si>
+    <t>https://www.boozallen.com/markets/defense/ai-for-military.html</t>
   </si>
 </sst>
 </file>
@@ -468,7 +489,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="47" customWidth="1"/>
@@ -558,6 +579,32 @@
         <v>22</v>
       </c>
     </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>